<commit_message>
feat(web): enhance seller panel for enterprise customers, sales, and data-table UX
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/customer-import-template.xlsx
+++ b/apps/web/public/templates/customer-import-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>phone</t>
   </si>
@@ -22,19 +22,61 @@
     <t>local_code</t>
   </si>
   <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>national_id</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>tags</t>
+  </si>
+  <si>
+    <t>address_line</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>phone2</t>
+  </si>
+  <si>
+    <t>emergency_name</t>
+  </si>
+  <si>
+    <t>emergency_phone</t>
+  </si>
+  <si>
     <t>notes</t>
   </si>
   <si>
     <t>09121234567</t>
   </si>
   <si>
-    <t>حسین احمدی</t>
+    <t>علی رضایی</t>
   </si>
   <si>
     <t>C-001</t>
   </si>
   <si>
-    <t>مشتری قدیمی</t>
+    <t>ali@example.com</t>
+  </si>
+  <si>
+    <t>1234567890</t>
+  </si>
+  <si>
+    <t>vip</t>
+  </si>
+  <si>
+    <t>vip,regular</t>
+  </si>
+  <si>
+    <t>خیابان آزادی ۱۲</t>
+  </si>
+  <si>
+    <t>تهران</t>
   </si>
   <si>
     <t>09129876543</t>
@@ -43,20 +85,26 @@
     <t>مریم رضایی</t>
   </si>
   <si>
-    <t/>
+    <t>09121112222</t>
+  </si>
+  <si>
+    <t>یادداشت نمونه</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -79,8 +127,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -420,49 +471,104 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="21" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>